<commit_message>
agregada la función de enviar via whatsapp
</commit_message>
<xml_diff>
--- a/Plantilla/Ventas_Marzo_Informe_Automatico.xlsx
+++ b/Plantilla/Ventas_Marzo_Informe_Automatico.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="5" activeTab="10" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Datos" sheetId="1" state="visible" r:id="rId1"/>
@@ -1428,19 +1428,46 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1449,93 +1476,66 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="27" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="44" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="46" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="29" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="39" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="49" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="43" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="45" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="47" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="48" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="40" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="42" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="44" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="46" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="32" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1569,49 +1569,49 @@
     <xf numFmtId="0" fontId="55" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="59" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="57" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="59" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="62" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="57" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="60" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="58" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="61" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="32" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="62" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="60" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="61" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="65" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="63" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="64" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="63" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="32" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -2467,10 +2467,10 @@
         </is>
       </c>
       <c r="C2" s="198" t="n">
-        <v>4268013.2768</v>
+        <v>4590909.090909091</v>
       </c>
       <c r="D2" s="12" t="n">
-        <v>223580</v>
+        <v>3507906</v>
       </c>
       <c r="E2" s="13">
         <f>D2/C2</f>
@@ -2480,7 +2480,7 @@
         <v>15</v>
       </c>
       <c r="G2" s="14" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H2" s="15">
         <f>G2/F2</f>
@@ -2513,10 +2513,10 @@
         </is>
       </c>
       <c r="C3" s="201" t="n">
-        <v>5782400</v>
+        <v>6500000</v>
       </c>
       <c r="D3" s="21" t="n">
-        <v>2028947</v>
+        <v>2855804</v>
       </c>
       <c r="E3" s="22">
         <f>D3/C3</f>
@@ -2536,7 +2536,7 @@
         <f>F3-G3</f>
         <v/>
       </c>
-      <c r="J3" s="134" t="n"/>
+      <c r="J3" s="135" t="n"/>
       <c r="K3">
         <f>IFERROR(VLOOKUP(B3,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2556,10 +2556,10 @@
         </is>
       </c>
       <c r="C4" s="198" t="n">
-        <v>3912073.134342516</v>
+        <v>4181818.181818182</v>
       </c>
       <c r="D4" s="12" t="n">
-        <v>685009</v>
+        <v>2045015</v>
       </c>
       <c r="E4" s="13">
         <f>D4/C4</f>
@@ -2569,7 +2569,7 @@
         <v>35</v>
       </c>
       <c r="G4" s="14" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="H4" s="15">
         <f>G4/F4</f>
@@ -2602,10 +2602,10 @@
         </is>
       </c>
       <c r="C5" s="202" t="n">
-        <v>3557632.361851224</v>
+        <v>3954545.454545455</v>
       </c>
       <c r="D5" s="29" t="n">
-        <v>351601</v>
+        <v>2339399</v>
       </c>
       <c r="E5" s="30">
         <f>D5/C5</f>
@@ -2615,7 +2615,7 @@
         <v>35</v>
       </c>
       <c r="G5" s="31" t="n">
-        <v>5</v>
+        <v>28</v>
       </c>
       <c r="H5" s="32">
         <f>G5/F5</f>
@@ -2625,7 +2625,7 @@
         <f>F5-G5</f>
         <v/>
       </c>
-      <c r="J5" s="135" t="n"/>
+      <c r="J5" s="134" t="n"/>
       <c r="K5">
         <f>IFERROR(VLOOKUP(B5,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2645,10 +2645,10 @@
         </is>
       </c>
       <c r="C6" s="203" t="n">
-        <v>4352260.401763355</v>
+        <v>4500000</v>
       </c>
       <c r="D6" s="36" t="n">
-        <v>1022481</v>
+        <v>2678605</v>
       </c>
       <c r="E6" s="37">
         <f>D6/C6</f>
@@ -2658,7 +2658,7 @@
         <v>25</v>
       </c>
       <c r="G6" s="38" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="H6" s="39">
         <f>G6/F6</f>
@@ -2668,7 +2668,7 @@
         <f>F6-G6</f>
         <v/>
       </c>
-      <c r="J6" s="135" t="n"/>
+      <c r="J6" s="134" t="n"/>
       <c r="K6">
         <f>IFERROR(VLOOKUP(B6,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2688,10 +2688,10 @@
         </is>
       </c>
       <c r="C7" s="203" t="n">
-        <v>2949191.375180122</v>
+        <v>3454545.454545455</v>
       </c>
       <c r="D7" s="36" t="n">
-        <v>2255194</v>
+        <v>2554479</v>
       </c>
       <c r="E7" s="37">
         <f>D7/C7</f>
@@ -2701,7 +2701,7 @@
         <v>35</v>
       </c>
       <c r="G7" s="38" t="n">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="H7" s="39">
         <f>G7/F7</f>
@@ -2711,7 +2711,7 @@
         <f>F7-G7</f>
         <v/>
       </c>
-      <c r="J7" s="135" t="n"/>
+      <c r="J7" s="134" t="n"/>
       <c r="K7">
         <f>IFERROR(VLOOKUP(B7,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2731,10 +2731,10 @@
         </is>
       </c>
       <c r="C8" s="202" t="n">
-        <v>3599832.422679558</v>
+        <v>3909090.909090909</v>
       </c>
       <c r="D8" s="29" t="n">
-        <v>526457</v>
+        <v>2089734</v>
       </c>
       <c r="E8" s="30">
         <f>D8/C8</f>
@@ -2744,7 +2744,7 @@
         <v>35</v>
       </c>
       <c r="G8" s="31" t="n">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="H8" s="32">
         <f>G8/F8</f>
@@ -2754,7 +2754,7 @@
         <f>F8-G8</f>
         <v/>
       </c>
-      <c r="J8" s="135" t="n"/>
+      <c r="J8" s="134" t="n"/>
       <c r="K8">
         <f>IFERROR(VLOOKUP(B8,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2774,10 +2774,10 @@
         </is>
       </c>
       <c r="C9" s="202" t="n">
-        <v>4051883.292469844</v>
+        <v>4972102.727272728</v>
       </c>
       <c r="D9" s="29" t="n">
-        <v>3112600</v>
+        <v>1534171</v>
       </c>
       <c r="E9" s="30">
         <f>D9/C9</f>
@@ -2787,7 +2787,7 @@
         <v>25</v>
       </c>
       <c r="G9" s="31" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H9" s="32">
         <f>G9/F9</f>
@@ -2797,7 +2797,7 @@
         <f>F9-G9</f>
         <v/>
       </c>
-      <c r="J9" s="135" t="n"/>
+      <c r="J9" s="134" t="n"/>
       <c r="K9">
         <f>IFERROR(VLOOKUP(B9,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2817,10 +2817,10 @@
         </is>
       </c>
       <c r="C10" s="202" t="n">
-        <v>4501003.655035949</v>
+        <v>4727272.727272728</v>
       </c>
       <c r="D10" s="29" t="n">
-        <v>1633262</v>
+        <v>2044715</v>
       </c>
       <c r="E10" s="30">
         <f>D10/C10</f>
@@ -2830,7 +2830,7 @@
         <v>35</v>
       </c>
       <c r="G10" s="31" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H10" s="32">
         <f>G10/F10</f>
@@ -2840,7 +2840,7 @@
         <f>F10-G10</f>
         <v/>
       </c>
-      <c r="J10" s="135" t="n"/>
+      <c r="J10" s="134" t="n"/>
       <c r="K10">
         <f>IFERROR(VLOOKUP(B10,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2860,10 +2860,10 @@
         </is>
       </c>
       <c r="C11" s="201" t="n">
-        <v>4068123.345954158</v>
+        <v>4022727.272727273</v>
       </c>
       <c r="D11" s="21" t="n">
-        <v>394472</v>
+        <v>1721783</v>
       </c>
       <c r="E11" s="22">
         <f>D11/C11</f>
@@ -2873,7 +2873,7 @@
         <v>35</v>
       </c>
       <c r="G11" s="23" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H11" s="24">
         <f>G11/F11</f>
@@ -2883,7 +2883,7 @@
         <f>F11-G11</f>
         <v/>
       </c>
-      <c r="J11" s="134" t="n"/>
+      <c r="J11" s="135" t="n"/>
       <c r="K11">
         <f>IFERROR(VLOOKUP(B11,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2903,10 +2903,10 @@
         </is>
       </c>
       <c r="C12" s="198" t="n">
-        <v>2115234.39982896</v>
+        <v>2227272.727272727</v>
       </c>
       <c r="D12" s="12" t="n">
-        <v>73431</v>
+        <v>1176010</v>
       </c>
       <c r="E12" s="13">
         <f>D12/C12</f>
@@ -2916,7 +2916,7 @@
         <v>35</v>
       </c>
       <c r="G12" s="14" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="H12" s="15">
         <f>G12/F12</f>
@@ -2949,10 +2949,10 @@
         </is>
       </c>
       <c r="C13" s="202" t="n">
-        <v>2350449.421398123</v>
+        <v>2622727.272727273</v>
       </c>
       <c r="D13" s="29" t="n">
-        <v>1408251</v>
+        <v>1102811</v>
       </c>
       <c r="E13" s="30">
         <f>D13/C13</f>
@@ -2962,7 +2962,7 @@
         <v>35</v>
       </c>
       <c r="G13" s="31" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="H13" s="32">
         <f>G13/F13</f>
@@ -2972,7 +2972,7 @@
         <f>F13-G13</f>
         <v/>
       </c>
-      <c r="J13" s="135" t="n"/>
+      <c r="J13" s="134" t="n"/>
       <c r="K13">
         <f>IFERROR(VLOOKUP(B13,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -2992,10 +2992,10 @@
         </is>
       </c>
       <c r="C14" s="202" t="n">
-        <v>2027779.239515265</v>
+        <v>2059090.909090909</v>
       </c>
       <c r="D14" s="29" t="n">
-        <v>519632</v>
+        <v>637691</v>
       </c>
       <c r="E14" s="30">
         <f>D14/C14</f>
@@ -3005,7 +3005,7 @@
         <v>35</v>
       </c>
       <c r="G14" s="31" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H14" s="32">
         <f>G14/F14</f>
@@ -3015,7 +3015,7 @@
         <f>F14-G14</f>
         <v/>
       </c>
-      <c r="J14" s="135" t="n"/>
+      <c r="J14" s="134" t="n"/>
       <c r="K14">
         <f>IFERROR(VLOOKUP(B14,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3035,10 +3035,10 @@
         </is>
       </c>
       <c r="C15" s="202" t="n">
-        <v>1995472.141940475</v>
+        <v>1909090.909090909</v>
       </c>
       <c r="D15" s="29" t="n">
-        <v>526732</v>
+        <v>1993218</v>
       </c>
       <c r="E15" s="30">
         <f>D15/C15</f>
@@ -3048,7 +3048,7 @@
         <v>35</v>
       </c>
       <c r="G15" s="31" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
       <c r="H15" s="32">
         <f>G15/F15</f>
@@ -3058,7 +3058,7 @@
         <f>F15-G15</f>
         <v/>
       </c>
-      <c r="J15" s="135" t="n"/>
+      <c r="J15" s="134" t="n"/>
       <c r="K15">
         <f>IFERROR(VLOOKUP(B15,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3078,10 +3078,10 @@
         </is>
       </c>
       <c r="C16" s="203" t="n">
-        <v>2883608.019584803</v>
+        <v>3522727.272727273</v>
       </c>
       <c r="D16" s="36" t="n">
-        <v>1574351</v>
+        <v>1051578</v>
       </c>
       <c r="E16" s="37">
         <f>D16/C16</f>
@@ -3091,7 +3091,7 @@
         <v>25</v>
       </c>
       <c r="G16" s="38" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="H16" s="39">
         <f>G16/F16</f>
@@ -3101,7 +3101,7 @@
         <f>F16-G16</f>
         <v/>
       </c>
-      <c r="J16" s="135" t="n"/>
+      <c r="J16" s="134" t="n"/>
       <c r="K16">
         <f>IFERROR(VLOOKUP(B16,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3121,10 +3121,10 @@
         </is>
       </c>
       <c r="C17" s="202" t="n">
-        <v>2192336.459053269</v>
+        <v>2590909.090909091</v>
       </c>
       <c r="D17" s="29" t="n">
-        <v>1300154</v>
+        <v>890550</v>
       </c>
       <c r="E17" s="30">
         <f>D17/C17</f>
@@ -3144,7 +3144,7 @@
         <f>F17-G17</f>
         <v/>
       </c>
-      <c r="J17" s="135" t="n"/>
+      <c r="J17" s="134" t="n"/>
       <c r="K17">
         <f>IFERROR(VLOOKUP(B17,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3164,10 +3164,10 @@
         </is>
       </c>
       <c r="C18" s="203" t="n">
-        <v>2822450.21446998</v>
+        <v>3250000</v>
       </c>
       <c r="D18" s="36" t="n">
-        <v>1744705</v>
+        <v>1417935</v>
       </c>
       <c r="E18" s="37">
         <f>D18/C18</f>
@@ -3177,7 +3177,7 @@
         <v>25</v>
       </c>
       <c r="G18" s="38" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H18" s="39">
         <f>G18/F18</f>
@@ -3187,7 +3187,7 @@
         <f>F18-G18</f>
         <v/>
       </c>
-      <c r="J18" s="135" t="n"/>
+      <c r="J18" s="134" t="n"/>
       <c r="K18">
         <f>IFERROR(VLOOKUP(B18,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3207,10 +3207,10 @@
         </is>
       </c>
       <c r="C19" s="201" t="n">
-        <v>1875070.115217594</v>
+        <v>2090909.090909091</v>
       </c>
       <c r="D19" s="21" t="n">
-        <v>591233</v>
+        <v>1023986</v>
       </c>
       <c r="E19" s="22">
         <f>D19/C19</f>
@@ -3220,7 +3220,7 @@
         <v>35</v>
       </c>
       <c r="G19" s="23" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="H19" s="24">
         <f>G19/F19</f>
@@ -3230,7 +3230,7 @@
         <f>F19-G19</f>
         <v/>
       </c>
-      <c r="J19" s="134" t="n"/>
+      <c r="J19" s="135" t="n"/>
       <c r="K19">
         <f>IFERROR(VLOOKUP(B19,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3250,10 +3250,10 @@
         </is>
       </c>
       <c r="C20" s="198" t="n">
-        <v>3489091.338384212</v>
+        <v>3345454.545454545</v>
       </c>
       <c r="D20" s="12" t="n">
-        <v>984789</v>
+        <v>1863599</v>
       </c>
       <c r="E20" s="13">
         <f>D20/C20</f>
@@ -3263,7 +3263,7 @@
         <v>35</v>
       </c>
       <c r="G20" s="14" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="H20" s="15">
         <f>G20/F20</f>
@@ -3296,10 +3296,10 @@
         </is>
       </c>
       <c r="C21" s="202" t="n">
-        <v>2577874.325332872</v>
+        <v>3690939.545454545</v>
       </c>
       <c r="D21" s="29" t="n">
-        <v>583371</v>
+        <v>1122040</v>
       </c>
       <c r="E21" s="30">
         <f>D21/C21</f>
@@ -3309,7 +3309,7 @@
         <v>35</v>
       </c>
       <c r="G21" s="31" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="H21" s="32">
         <f>G21/F21</f>
@@ -3319,7 +3319,7 @@
         <f>F21-G21</f>
         <v/>
       </c>
-      <c r="J21" s="135" t="n"/>
+      <c r="J21" s="134" t="n"/>
       <c r="K21">
         <f>IFERROR(VLOOKUP(B21,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3339,10 +3339,10 @@
         </is>
       </c>
       <c r="C22" s="202" t="n">
-        <v>4147681.156904749</v>
+        <v>5454545.454545454</v>
       </c>
       <c r="D22" s="29" t="n">
-        <v>3327707</v>
+        <v>1588813</v>
       </c>
       <c r="E22" s="30">
         <f>D22/C22</f>
@@ -3352,7 +3352,7 @@
         <v>25</v>
       </c>
       <c r="G22" s="31" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H22" s="32">
         <f>G22/F22</f>
@@ -3362,7 +3362,7 @@
         <f>F22-G22</f>
         <v/>
       </c>
-      <c r="J22" s="135" t="n"/>
+      <c r="J22" s="134" t="n"/>
       <c r="K22">
         <f>IFERROR(VLOOKUP(B22,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3382,10 +3382,10 @@
         </is>
       </c>
       <c r="C23" s="202" t="n">
-        <v>2540205.099875077</v>
+        <v>2568181.818181818</v>
       </c>
       <c r="D23" s="29" t="n">
-        <v>784817</v>
+        <v>1208014</v>
       </c>
       <c r="E23" s="30">
         <f>D23/C23</f>
@@ -3395,7 +3395,7 @@
         <v>35</v>
       </c>
       <c r="G23" s="31" t="n">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="H23" s="32">
         <f>G23/F23</f>
@@ -3405,7 +3405,7 @@
         <f>F23-G23</f>
         <v/>
       </c>
-      <c r="J23" s="135" t="n"/>
+      <c r="J23" s="134" t="n"/>
       <c r="K23">
         <f>IFERROR(VLOOKUP(B23,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3425,10 +3425,10 @@
         </is>
       </c>
       <c r="C24" s="203" t="n">
-        <v>3542990.117460595</v>
+        <v>4681818.181818182</v>
       </c>
       <c r="D24" s="36" t="n">
-        <v>2322726</v>
+        <v>3866287</v>
       </c>
       <c r="E24" s="37">
         <f>D24/C24</f>
@@ -3438,7 +3438,7 @@
         <v>25</v>
       </c>
       <c r="G24" s="38" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="H24" s="39">
         <f>G24/F24</f>
@@ -3448,7 +3448,7 @@
         <f>F24-G24</f>
         <v/>
       </c>
-      <c r="J24" s="135" t="n"/>
+      <c r="J24" s="134" t="n"/>
       <c r="K24">
         <f>IFERROR(VLOOKUP(B24,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3468,10 +3468,10 @@
         </is>
       </c>
       <c r="C25" s="203" t="n">
-        <v>2920413.487096615</v>
+        <v>2945454.545454545</v>
       </c>
       <c r="D25" s="36" t="n">
-        <v>869025</v>
+        <v>1219159</v>
       </c>
       <c r="E25" s="37">
         <f>D25/C25</f>
@@ -3481,7 +3481,7 @@
         <v>35</v>
       </c>
       <c r="G25" s="38" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H25" s="39">
         <f>G25/F25</f>
@@ -3491,7 +3491,7 @@
         <f>F25-G25</f>
         <v/>
       </c>
-      <c r="J25" s="135" t="n"/>
+      <c r="J25" s="134" t="n"/>
       <c r="K25">
         <f>IFERROR(VLOOKUP(B25,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3511,10 +3511,10 @@
         </is>
       </c>
       <c r="C26" s="202" t="n">
-        <v>2415122.61409575</v>
+        <v>2750000</v>
       </c>
       <c r="D26" s="29" t="n">
-        <v>415912</v>
+        <v>1522295</v>
       </c>
       <c r="E26" s="30">
         <f>D26/C26</f>
@@ -3524,7 +3524,7 @@
         <v>35</v>
       </c>
       <c r="G26" s="31" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="H26" s="32">
         <f>G26/F26</f>
@@ -3534,7 +3534,7 @@
         <f>F26-G26</f>
         <v/>
       </c>
-      <c r="J26" s="135" t="n"/>
+      <c r="J26" s="134" t="n"/>
       <c r="K26">
         <f>IFERROR(VLOOKUP(B26,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3554,10 +3554,10 @@
         </is>
       </c>
       <c r="C27" s="201" t="n">
-        <v>4616221.860850123</v>
+        <v>4545454.545454546</v>
       </c>
       <c r="D27" s="21" t="n">
-        <v>1920217</v>
+        <v>3556279</v>
       </c>
       <c r="E27" s="22">
         <f>D27/C27</f>
@@ -3567,7 +3567,7 @@
         <v>35</v>
       </c>
       <c r="G27" s="23" t="n">
-        <v>8</v>
+        <v>21</v>
       </c>
       <c r="H27" s="24">
         <f>G27/F27</f>
@@ -3577,7 +3577,7 @@
         <f>F27-G27</f>
         <v/>
       </c>
-      <c r="J27" s="134" t="n"/>
+      <c r="J27" s="135" t="n"/>
       <c r="K27">
         <f>IFERROR(VLOOKUP(B27,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3597,10 +3597,10 @@
         </is>
       </c>
       <c r="C28" s="198" t="n">
-        <v>2620062.334559925</v>
+        <v>2404545.454545455</v>
       </c>
       <c r="D28" s="12" t="n">
-        <v>562800</v>
+        <v>1002965</v>
       </c>
       <c r="E28" s="13">
         <f>D28/C28</f>
@@ -3610,7 +3610,7 @@
         <v>35</v>
       </c>
       <c r="G28" s="14" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="H28" s="15">
         <f>G28/F28</f>
@@ -3643,10 +3643,10 @@
         </is>
       </c>
       <c r="C29" s="202" t="n">
-        <v>2458438.608382704</v>
+        <v>2822727.272727273</v>
       </c>
       <c r="D29" s="29" t="n">
-        <v>915675</v>
+        <v>1488895</v>
       </c>
       <c r="E29" s="30">
         <f>D29/C29</f>
@@ -3656,7 +3656,7 @@
         <v>35</v>
       </c>
       <c r="G29" s="31" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="H29" s="32">
         <f>G29/F29</f>
@@ -3666,7 +3666,7 @@
         <f>F29-G29</f>
         <v/>
       </c>
-      <c r="J29" s="135" t="n"/>
+      <c r="J29" s="134" t="n"/>
       <c r="K29">
         <f>IFERROR(VLOOKUP(B29,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3686,10 +3686,10 @@
         </is>
       </c>
       <c r="C30" s="203" t="n">
-        <v>2514139.040663015</v>
+        <v>3131818.181818182</v>
       </c>
       <c r="D30" s="36" t="n">
-        <v>2400108</v>
+        <v>1269089</v>
       </c>
       <c r="E30" s="37">
         <f>D30/C30</f>
@@ -3699,7 +3699,7 @@
         <v>25</v>
       </c>
       <c r="G30" s="38" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H30" s="39">
         <f>G30/F30</f>
@@ -3709,7 +3709,7 @@
         <f>F30-G30</f>
         <v/>
       </c>
-      <c r="J30" s="135" t="n"/>
+      <c r="J30" s="134" t="n"/>
       <c r="K30">
         <f>IFERROR(VLOOKUP(B30,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3729,10 +3729,10 @@
         </is>
       </c>
       <c r="C31" s="202" t="n">
-        <v>2647652.665731449</v>
+        <v>2909090.909090909</v>
       </c>
       <c r="D31" s="29" t="n">
-        <v>135262</v>
+        <v>2485159</v>
       </c>
       <c r="E31" s="30">
         <f>D31/C31</f>
@@ -3742,7 +3742,7 @@
         <v>35</v>
       </c>
       <c r="G31" s="31" t="n">
-        <v>2</v>
+        <v>39</v>
       </c>
       <c r="H31" s="32">
         <f>G31/F31</f>
@@ -3752,7 +3752,7 @@
         <f>F31-G31</f>
         <v/>
       </c>
-      <c r="J31" s="135" t="n"/>
+      <c r="J31" s="134" t="n"/>
       <c r="K31">
         <f>IFERROR(VLOOKUP(B31,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3772,10 +3772,10 @@
         </is>
       </c>
       <c r="C32" s="202" t="n">
-        <v>2470680.767831972</v>
+        <v>2477272.727272727</v>
       </c>
       <c r="D32" s="29" t="n">
-        <v>64164</v>
+        <v>1377308</v>
       </c>
       <c r="E32" s="30">
         <f>D32/C32</f>
@@ -3785,7 +3785,7 @@
         <v>35</v>
       </c>
       <c r="G32" s="31" t="n">
-        <v>3</v>
+        <v>24</v>
       </c>
       <c r="H32" s="32">
         <f>G32/F32</f>
@@ -3795,7 +3795,7 @@
         <f>F32-G32</f>
         <v/>
       </c>
-      <c r="J32" s="135" t="n"/>
+      <c r="J32" s="134" t="n"/>
       <c r="K32">
         <f>IFERROR(VLOOKUP(B32,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3815,10 +3815,10 @@
         </is>
       </c>
       <c r="C33" s="203" t="n">
-        <v>2270254.174878573</v>
+        <v>2631818.181818182</v>
       </c>
       <c r="D33" s="36" t="n">
-        <v>1483330</v>
+        <v>1064054</v>
       </c>
       <c r="E33" s="37">
         <f>D33/C33</f>
@@ -3828,7 +3828,7 @@
         <v>25</v>
       </c>
       <c r="G33" s="38" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H33" s="39">
         <f>G33/F33</f>
@@ -3838,7 +3838,7 @@
         <f>F33-G33</f>
         <v/>
       </c>
-      <c r="J33" s="135" t="n"/>
+      <c r="J33" s="134" t="n"/>
       <c r="K33">
         <f>IFERROR(VLOOKUP(B33,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3858,10 +3858,10 @@
         </is>
       </c>
       <c r="C34" s="202" t="n">
-        <v>2328805.581573491</v>
+        <v>2363636.363636364</v>
       </c>
       <c r="D34" s="29" t="n">
-        <v>296644</v>
+        <v>1629772</v>
       </c>
       <c r="E34" s="30">
         <f>D34/C34</f>
@@ -3871,7 +3871,7 @@
         <v>35</v>
       </c>
       <c r="G34" s="31" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="H34" s="32">
         <f>G34/F34</f>
@@ -3881,7 +3881,7 @@
         <f>F34-G34</f>
         <v/>
       </c>
-      <c r="J34" s="135" t="n"/>
+      <c r="J34" s="134" t="n"/>
       <c r="K34">
         <f>IFERROR(VLOOKUP(B34,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3901,10 +3901,10 @@
         </is>
       </c>
       <c r="C35" s="201" t="n">
-        <v>1534766.807726665</v>
+        <v>2431818.181818182</v>
       </c>
       <c r="D35" s="21" t="n">
-        <v>49563</v>
+        <v>1470596</v>
       </c>
       <c r="E35" s="22">
         <f>D35/C35</f>
@@ -3914,7 +3914,7 @@
         <v>35</v>
       </c>
       <c r="G35" s="23" t="n">
-        <v>2</v>
+        <v>19</v>
       </c>
       <c r="H35" s="24">
         <f>G35/F35</f>
@@ -3924,7 +3924,7 @@
         <f>F35-G35</f>
         <v/>
       </c>
-      <c r="J35" s="134" t="n"/>
+      <c r="J35" s="135" t="n"/>
       <c r="K35">
         <f>IFERROR(VLOOKUP(B35,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -3944,10 +3944,10 @@
         </is>
       </c>
       <c r="C36" s="204" t="n">
-        <v>14768000</v>
+        <v>17727272.72727273</v>
       </c>
       <c r="D36" s="44" t="n">
-        <v>8856753</v>
+        <v>3320656</v>
       </c>
       <c r="E36" s="45">
         <f>D36/C36</f>
@@ -3957,7 +3957,7 @@
         <v>10</v>
       </c>
       <c r="G36" s="46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H36" s="47">
         <f>G36/F36</f>
@@ -3990,10 +3990,10 @@
         </is>
       </c>
       <c r="C37" s="198" t="n">
-        <v>744134.1856</v>
+        <v>795454.5454545454</v>
       </c>
       <c r="D37" s="12" t="n">
-        <v>144725</v>
+        <v>203130</v>
       </c>
       <c r="E37" s="13">
         <f>D37/C37</f>
@@ -4003,7 +4003,7 @@
         <v>25</v>
       </c>
       <c r="G37" s="14" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="H37" s="15">
         <f>G37/F37</f>
@@ -4036,10 +4036,10 @@
         </is>
       </c>
       <c r="C38" s="202" t="n">
-        <v>744134.1856</v>
+        <v>795454.5454545454</v>
       </c>
       <c r="D38" s="29" t="n">
-        <v>135701</v>
+        <v>789621</v>
       </c>
       <c r="E38" s="30">
         <f>D38/C38</f>
@@ -4049,7 +4049,7 @@
         <v>25</v>
       </c>
       <c r="G38" s="31" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="H38" s="32">
         <f>G38/F38</f>
@@ -4059,7 +4059,7 @@
         <f>F38-G38</f>
         <v/>
       </c>
-      <c r="J38" s="135" t="n"/>
+      <c r="J38" s="134" t="n"/>
       <c r="K38">
         <f>IFERROR(VLOOKUP(B38,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4079,10 +4079,10 @@
         </is>
       </c>
       <c r="C39" s="202" t="n">
-        <v>744134.1856</v>
+        <v>795454.5454545454</v>
       </c>
       <c r="D39" s="29" t="n">
-        <v>150873</v>
+        <v>548468</v>
       </c>
       <c r="E39" s="30">
         <f>D39/C39</f>
@@ -4092,7 +4092,7 @@
         <v>25</v>
       </c>
       <c r="G39" s="31" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="H39" s="32">
         <f>G39/F39</f>
@@ -4102,7 +4102,7 @@
         <f>F39-G39</f>
         <v/>
       </c>
-      <c r="J39" s="135" t="n"/>
+      <c r="J39" s="134" t="n"/>
       <c r="K39">
         <f>IFERROR(VLOOKUP(B39,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4122,10 +4122,10 @@
         </is>
       </c>
       <c r="C40" s="202" t="n">
-        <v>744134.1856</v>
+        <v>795454.5454545454</v>
       </c>
       <c r="D40" s="29" t="n">
-        <v>76728</v>
+        <v>625620</v>
       </c>
       <c r="E40" s="30">
         <f>D40/C40</f>
@@ -4135,7 +4135,7 @@
         <v>25</v>
       </c>
       <c r="G40" s="31" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="H40" s="32">
         <f>G40/F40</f>
@@ -4145,7 +4145,7 @@
         <f>F40-G40</f>
         <v/>
       </c>
-      <c r="J40" s="135" t="n"/>
+      <c r="J40" s="134" t="n"/>
       <c r="K40">
         <f>IFERROR(VLOOKUP(B40,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4165,10 +4165,10 @@
         </is>
       </c>
       <c r="C41" s="202" t="n">
-        <v>744134.1856</v>
+        <v>795454.5454545454</v>
       </c>
       <c r="D41" s="29" t="n">
-        <v>2789524</v>
+        <v>334430</v>
       </c>
       <c r="E41" s="30">
         <f>D41/C41</f>
@@ -4178,7 +4178,7 @@
         <v>25</v>
       </c>
       <c r="G41" s="31" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="H41" s="32">
         <f>G41/F41</f>
@@ -4188,7 +4188,7 @@
         <f>F41-G41</f>
         <v/>
       </c>
-      <c r="J41" s="135" t="n"/>
+      <c r="J41" s="134" t="n"/>
       <c r="K41">
         <f>IFERROR(VLOOKUP(B41,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4208,10 +4208,10 @@
         </is>
       </c>
       <c r="C42" s="202" t="n">
-        <v>744134.1856</v>
+        <v>795454.5454545454</v>
       </c>
       <c r="D42" s="29" t="n">
-        <v>51687</v>
+        <v>488425</v>
       </c>
       <c r="E42" s="30">
         <f>D42/C42</f>
@@ -4221,7 +4221,7 @@
         <v>25</v>
       </c>
       <c r="G42" s="31" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="H42" s="32">
         <f>G42/F42</f>
@@ -4231,7 +4231,7 @@
         <f>F42-G42</f>
         <v/>
       </c>
-      <c r="J42" s="135" t="n"/>
+      <c r="J42" s="134" t="n"/>
       <c r="K42">
         <f>IFERROR(VLOOKUP(B42,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4251,10 +4251,10 @@
         </is>
       </c>
       <c r="C43" s="203" t="n">
-        <v>893894.1856</v>
+        <v>1704066.136363636</v>
       </c>
       <c r="D43" s="36" t="n">
-        <v>5248333</v>
+        <v>436523</v>
       </c>
       <c r="E43" s="37">
         <f>D43/C43</f>
@@ -4264,7 +4264,7 @@
         <v>20</v>
       </c>
       <c r="G43" s="38" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="H43" s="39">
         <f>G43/F43</f>
@@ -4274,7 +4274,7 @@
         <f>F43-G43</f>
         <v/>
       </c>
-      <c r="J43" s="135" t="n"/>
+      <c r="J43" s="134" t="n"/>
       <c r="K43">
         <f>IFERROR(VLOOKUP(B43,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4294,10 +4294,10 @@
         </is>
       </c>
       <c r="C44" s="205" t="n">
-        <v>893894.1439999999</v>
+        <v>1704066.136363636</v>
       </c>
       <c r="D44" s="51" t="n">
-        <v>511650</v>
+        <v>289338</v>
       </c>
       <c r="E44" s="52">
         <f>D44/C44</f>
@@ -4307,7 +4307,7 @@
         <v>20</v>
       </c>
       <c r="G44" s="53" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H44" s="54">
         <f>G44/F44</f>
@@ -4317,7 +4317,7 @@
         <f>F44-G44</f>
         <v/>
       </c>
-      <c r="J44" s="134" t="n"/>
+      <c r="J44" s="135" t="n"/>
       <c r="K44">
         <f>IFERROR(VLOOKUP(B44,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4337,10 +4337,10 @@
         </is>
       </c>
       <c r="C45" s="206" t="n">
-        <v>2356623.36</v>
+        <v>2634545.454545454</v>
       </c>
       <c r="D45" s="58" t="n">
-        <v>399745</v>
+        <v>1489725</v>
       </c>
       <c r="E45" s="59">
         <f>D45/C45</f>
@@ -4350,7 +4350,7 @@
         <v>42</v>
       </c>
       <c r="G45" s="60" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="H45" s="61">
         <f>G45/F45</f>
@@ -4383,10 +4383,10 @@
         </is>
       </c>
       <c r="C46" s="202" t="n">
-        <v>1876992</v>
+        <v>2409090.909090909</v>
       </c>
       <c r="D46" s="29" t="n">
-        <v>387831</v>
+        <v>1098479</v>
       </c>
       <c r="E46" s="30">
         <f>D46/C46</f>
@@ -4396,7 +4396,7 @@
         <v>42</v>
       </c>
       <c r="G46" s="31" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="H46" s="32">
         <f>G46/F46</f>
@@ -4406,7 +4406,7 @@
         <f>F46-G46</f>
         <v/>
       </c>
-      <c r="J46" s="135" t="n"/>
+      <c r="J46" s="134" t="n"/>
       <c r="K46">
         <f>IFERROR(VLOOKUP(B46,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4426,10 +4426,10 @@
         </is>
       </c>
       <c r="C47" s="202" t="n">
-        <v>3320977.92</v>
+        <v>3753818.181818182</v>
       </c>
       <c r="D47" s="29" t="n">
-        <v>725808</v>
+        <v>373011</v>
       </c>
       <c r="E47" s="30">
         <f>D47/C47</f>
@@ -4439,7 +4439,7 @@
         <v>42</v>
       </c>
       <c r="G47" s="31" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H47" s="32">
         <f>G47/F47</f>
@@ -4449,7 +4449,7 @@
         <f>F47-G47</f>
         <v/>
       </c>
-      <c r="J47" s="135" t="n"/>
+      <c r="J47" s="134" t="n"/>
       <c r="K47">
         <f>IFERROR(VLOOKUP(B47,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4469,10 +4469,10 @@
         </is>
       </c>
       <c r="C48" s="202" t="n">
-        <v>2558400</v>
+        <v>2795454.545454545</v>
       </c>
       <c r="D48" s="29" t="n">
-        <v>1599658</v>
+        <v>1821028</v>
       </c>
       <c r="E48" s="30">
         <f>D48/C48</f>
@@ -4482,7 +4482,7 @@
         <v>42</v>
       </c>
       <c r="G48" s="31" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H48" s="32">
         <f>G48/F48</f>
@@ -4492,7 +4492,7 @@
         <f>F48-G48</f>
         <v/>
       </c>
-      <c r="J48" s="134" t="n"/>
+      <c r="J48" s="135" t="n"/>
       <c r="K48">
         <f>IFERROR(VLOOKUP(B48,[1]Hoja1!$A$4:$B$48,2,),0)</f>
         <v/>
@@ -4556,7 +4556,7 @@
         <f>F50-G50</f>
         <v/>
       </c>
-      <c r="J50" s="134" t="n"/>
+      <c r="J50" s="135" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -4594,7 +4594,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — COLOMBINA HELADOS</t>
         </is>
@@ -4611,41 +4611,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="188" t="inlineStr">
+      <c r="B6" s="192" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="191">
+      <c r="B7" s="190">
         <f>TEXT((Datos!D2+Datos!D3)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C2+Datos!C3)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D2+Datos!D3)/(Datos!C2+Datos!C3),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G2+Datos!G3)/(Datos!F2+Datos!F3),"0.0%")</f>
         <v/>
       </c>
@@ -4654,41 +4654,41 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
       </c>
-      <c r="F11" s="189" t="inlineStr">
+      <c r="F11" s="188" t="inlineStr">
         <is>
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G2+Datos!G3,"0")&amp;" / "&amp;TEXT(Datos!F2+Datos!F3,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H2:H3,"&gt;="&amp;1),"0")&amp;" / "&amp;"2"</f>
         <v/>
       </c>
-      <c r="F12" s="192">
+      <c r="F12" s="191">
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B2:B3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0)),4))),MID(INDEX(Datos!B2:B3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0)),6,100),INDEX(Datos!B2:B3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F2+Datos!F3-Datos!G2+Datos!G3),"0")&amp;IF(Datos!G2+Datos!G3&gt;=Datos!F2+Datos!F3," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -4697,49 +4697,49 @@
     <row r="14" ht="18" customHeight="1" s="137"/>
     <row r="15" ht="7.5" customHeight="1" s="137"/>
     <row r="16" ht="19.5" customHeight="1" s="137">
-      <c r="B16" s="190" t="inlineStr">
+      <c r="B16" s="189" t="inlineStr">
         <is>
           <t>DETALLE DE ASESORES — COLOMBINA HELADOS</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -4839,7 +4839,7 @@
         <f>Datos!F2+Datos!F3</f>
         <v/>
       </c>
-      <c r="H20" s="155">
+      <c r="H20" s="158">
         <f>SUM(H18:H19)</f>
         <v/>
       </c>
@@ -4850,32 +4850,32 @@
     </row>
     <row r="21" ht="7.5" customHeight="1" s="137"/>
     <row r="22" ht="18" customHeight="1" s="137">
-      <c r="B22" s="158" t="inlineStr">
+      <c r="B22" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="137">
-      <c r="B23" s="156">
+      <c r="B23" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D2+Datos!D3)/(Datos!C2+Datos!C3),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="137">
-      <c r="B24" s="153">
+      <c r="B24" s="170">
         <f>IF(COUNTIF(Datos!H2:H3,"&gt;="&amp;1)=2,"✔ "&amp;2&amp;" de 2 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G2+Datos!G3)-(Datos!F2+Datos!F3))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H2:H3,"&gt;="&amp;1)&amp;" de 2 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F2+Datos!F3)-(Datos!G2+Datos!G3))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="137">
-      <c r="B25" s="156">
+      <c r="B25" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B2:B3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0)),4))),MID(INDEX(Datos!B2:B3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0)),6,100),INDEX(Datos!B2:B3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0)))&amp;" con "&amp;TEXT(MAX(Datos!D2:D3),"$#,##0")&amp;" y "&amp;INDEX(Datos!G2:G3,MATCH(MAX(Datos!D2:D3),Datos!D2:D3,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="137">
-      <c r="B26" s="153">
+      <c r="B26" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B2:B3,MATCH(MIN(Datos!D2:D3),Datos!D2:D3,0)),4))),MID(INDEX(Datos!B2:B3,MATCH(MIN(Datos!D2:D3),Datos!D2:D3,0)),6,100),INDEX(Datos!B2:B3,MATCH(MIN(Datos!D2:D3),Datos!D2:D3,0)))&amp;" con "&amp;TEXT(MIN(Datos!D2:D3),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E2:E3),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -4932,7 +4932,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — ALIMENTOS POLAR</t>
         </is>
@@ -4949,41 +4949,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="193" t="inlineStr">
+      <c r="B6" s="197" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="196">
+      <c r="B7" s="195">
         <f>TEXT((Datos!D45+Datos!D46+Datos!D47+Datos!D48)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C45+Datos!C46+Datos!C47+Datos!C48)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D45+Datos!D46+Datos!D47+Datos!D48)/(Datos!C45+Datos!C46+Datos!C47+Datos!C48),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G45+Datos!G46+Datos!G47+Datos!G48)/(Datos!F45+Datos!F46+Datos!F47+Datos!F48),"0.0%")</f>
         <v/>
       </c>
@@ -4992,41 +4992,41 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
       </c>
-      <c r="F11" s="197" t="inlineStr">
+      <c r="F11" s="193" t="inlineStr">
         <is>
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G45+Datos!G46+Datos!G47+Datos!G48,"0")&amp;" / "&amp;TEXT(Datos!F45+Datos!F46+Datos!F47+Datos!F48,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H45:H48,"&gt;="&amp;1),"0")&amp;" / "&amp;"4"</f>
         <v/>
       </c>
-      <c r="F12" s="195">
+      <c r="F12" s="196">
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B45:B48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0)),4))),MID(INDEX(Datos!B45:B48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0)),6,100),INDEX(Datos!B45:B48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F45+Datos!F46+Datos!F47+Datos!F48-Datos!G45+Datos!G46+Datos!G47+Datos!G48),"0")&amp;IF(Datos!G45+Datos!G46+Datos!G47+Datos!G48&gt;=Datos!F45+Datos!F46+Datos!F47+Datos!F48," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -5042,42 +5042,42 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -5245,7 +5245,7 @@
         <f>Datos!F45+Datos!F46+Datos!F47+Datos!F48</f>
         <v/>
       </c>
-      <c r="H22" s="155">
+      <c r="H22" s="158">
         <f>SUM(H18:H21)</f>
         <v/>
       </c>
@@ -5256,32 +5256,32 @@
     </row>
     <row r="23" ht="7.5" customHeight="1" s="137"/>
     <row r="24" ht="18" customHeight="1" s="137">
-      <c r="B24" s="158" t="inlineStr">
+      <c r="B24" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="137">
-      <c r="B25" s="156">
+      <c r="B25" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D45+Datos!D46+Datos!D47+Datos!D48)/(Datos!C45+Datos!C46+Datos!C47+Datos!C48),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="137">
-      <c r="B26" s="153">
+      <c r="B26" s="170">
         <f>IF(COUNTIF(Datos!H45:H48,"&gt;="&amp;1)=4,"✔ "&amp;4&amp;" de 4 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G45+Datos!G46+Datos!G47+Datos!G48)-(Datos!F45+Datos!F46+Datos!F47+Datos!F48))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H45:H48,"&gt;="&amp;1)&amp;" de 4 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F45+Datos!F46+Datos!F47+Datos!F48)-(Datos!G45+Datos!G46+Datos!G47+Datos!G48))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="137">
-      <c r="B27" s="156">
+      <c r="B27" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B45:B48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0)),4))),MID(INDEX(Datos!B45:B48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0)),6,100),INDEX(Datos!B45:B48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0)))&amp;" con "&amp;TEXT(MAX(Datos!D45:D48),"$#,##0")&amp;" y "&amp;INDEX(Datos!G45:G48,MATCH(MAX(Datos!D45:D48),Datos!D45:D48,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="137">
-      <c r="B28" s="153">
+      <c r="B28" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B45:B48,MATCH(MIN(Datos!D45:D48),Datos!D45:D48,0)),4))),MID(INDEX(Datos!B45:B48,MATCH(MIN(Datos!D45:D48),Datos!D45:D48,0)),6,100),INDEX(Datos!B45:B48,MATCH(MIN(Datos!D45:D48),Datos!D45:D48,0)))&amp;" con "&amp;TEXT(MIN(Datos!D45:D48),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E45:E48),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -5338,7 +5338,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>RANKING DE ASESORES — VENTA DÍA</t>
         </is>
@@ -5354,42 +5354,42 @@
       </c>
     </row>
     <row r="5" ht="19.5" customHeight="1" s="137">
-      <c r="B5" s="145" t="inlineStr">
+      <c r="B5" s="141" t="inlineStr">
         <is>
           <t>Pos.</t>
         </is>
       </c>
-      <c r="C5" s="145" t="inlineStr">
+      <c r="C5" s="141" t="inlineStr">
         <is>
           <t>Asesor</t>
         </is>
       </c>
-      <c r="D5" s="145" t="inlineStr">
+      <c r="D5" s="141" t="inlineStr">
         <is>
           <t>Unidad de Negocio</t>
         </is>
       </c>
-      <c r="E5" s="145" t="inlineStr">
+      <c r="E5" s="141" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="F5" s="145" t="inlineStr">
+      <c r="F5" s="141" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="G5" s="145" t="inlineStr">
+      <c r="G5" s="141" t="inlineStr">
         <is>
           <t>Facturas</t>
         </is>
       </c>
-      <c r="H5" s="145" t="inlineStr">
+      <c r="H5" s="141" t="inlineStr">
         <is>
           <t>% Cumpl. Plan</t>
         </is>
       </c>
-      <c r="I5" s="145" t="inlineStr">
+      <c r="I5" s="141" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
@@ -6096,16 +6096,16 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="136" t="inlineStr">
-        <is>
-          <t>INFORME DE VENTAS — Abril 2025</t>
+      <c r="B1" s="147" t="inlineStr">
+        <is>
+          <t>INFORME DE VENTAS</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" s="137"/>
     <row r="3" ht="12" customHeight="1" s="137"/>
     <row r="4" ht="18" customHeight="1" s="137">
-      <c r="B4" s="142" t="inlineStr">
+      <c r="B4" s="151" t="inlineStr">
         <is>
           <t>Dirección Comercial  |  47 asesores activos  |  8 unidades de negocio</t>
         </is>
@@ -6113,41 +6113,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="15.75" customHeight="1" s="137">
-      <c r="B6" s="140" t="inlineStr">
+      <c r="B6" s="136" t="inlineStr">
         <is>
           <t>VENTA DÍA TOTAL</t>
         </is>
       </c>
-      <c r="D6" s="145" t="inlineStr">
+      <c r="D6" s="141" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="138" t="inlineStr">
+      <c r="F6" s="140" t="inlineStr">
         <is>
           <t>CUMPL. PRESUPUESTO</t>
         </is>
       </c>
-      <c r="H6" s="148" t="inlineStr">
+      <c r="H6" s="144" t="inlineStr">
         <is>
           <t>CUMPL. PLAN PEDIDOS</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="144">
+      <c r="B7" s="139">
         <f>TEXT(SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!D2:D49)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="139">
+      <c r="D7" s="148">
         <f>TEXT(SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!C2:C49)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="146">
+      <c r="F7" s="142">
         <f>TEXT(SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!D2:D49)/SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!C2:C49),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="141">
+      <c r="H7" s="150">
         <f>TEXT(SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!G2:G49)/SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!F2:F49),"0.0%")</f>
         <v/>
       </c>
@@ -6156,41 +6156,41 @@
     <row r="9"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="15.75" customHeight="1" s="137">
-      <c r="B11" s="149" t="inlineStr">
+      <c r="B11" s="145" t="inlineStr">
         <is>
           <t>FACTURAS EMITIDAS</t>
         </is>
       </c>
-      <c r="D11" s="138" t="inlineStr">
+      <c r="D11" s="140" t="inlineStr">
         <is>
           <t>ASESORES CUMPLEN META</t>
         </is>
       </c>
-      <c r="F11" s="140" t="inlineStr">
+      <c r="F11" s="136" t="inlineStr">
         <is>
           <t>MEJOR UN (VENTA DÍA)</t>
         </is>
       </c>
-      <c r="H11" s="138" t="inlineStr">
+      <c r="H11" s="140" t="inlineStr">
         <is>
           <t>UN CRÍTICA (CUMPL.)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="147">
+      <c r="B12" s="143">
         <f>TEXT(SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!G2:G49),"#,##0")&amp;" / "&amp;TEXT(SUMIF(Datos!A2:A49,"&lt;&gt;"&amp;"",Datos!F2:F49),"#,##0")</f>
         <v/>
       </c>
-      <c r="D12" s="151">
+      <c r="D12" s="149">
         <f>TEXT(COUNTIF(Datos!E2:E49,"&gt;="&amp;0.9),"0")&amp;" / "&amp;TEXT(COUNTA(Datos!B2:B49)-1,"0")</f>
         <v/>
       </c>
-      <c r="F12" s="150">
+      <c r="F12" s="146">
         <f>INDEX(Datos!A2:A49,MATCH(MAX(Datos!D2:D49),Datos!D2:D49,0))</f>
         <v/>
       </c>
-      <c r="H12" s="151">
+      <c r="H12" s="149">
         <f>INDEX(Datos!A2:A49,MATCH(MIN(Datos!E2:E49),Datos!E2:E49,0))</f>
         <v/>
       </c>
@@ -6199,49 +6199,49 @@
     <row r="14"/>
     <row r="15" ht="7.5" customHeight="1" s="137"/>
     <row r="16" ht="19.5" customHeight="1" s="137">
-      <c r="B16" s="143" t="inlineStr">
+      <c r="B16" s="138" t="inlineStr">
         <is>
           <t>RESUMEN POR UNIDAD DE NEGOCIO</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="140" t="inlineStr">
+      <c r="B17" s="136" t="inlineStr">
         <is>
           <t>Unidad de Negocio</t>
         </is>
       </c>
-      <c r="C17" s="140" t="inlineStr">
+      <c r="C17" s="136" t="inlineStr">
         <is>
           <t>Asesores</t>
         </is>
       </c>
-      <c r="D17" s="140" t="inlineStr">
+      <c r="D17" s="136" t="inlineStr">
         <is>
           <t>Presupuesto Día</t>
         </is>
       </c>
-      <c r="E17" s="140" t="inlineStr">
+      <c r="E17" s="136" t="inlineStr">
         <is>
           <t>Venta Día</t>
         </is>
       </c>
-      <c r="F17" s="140" t="inlineStr">
+      <c r="F17" s="136" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="G17" s="140" t="inlineStr">
+      <c r="G17" s="136" t="inlineStr">
         <is>
           <t>Facturas</t>
         </is>
       </c>
-      <c r="H17" s="140" t="inlineStr">
+      <c r="H17" s="136" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="I17" s="140" t="inlineStr">
+      <c r="I17" s="136" t="inlineStr">
         <is>
           <t>% Cumpl. Plan</t>
         </is>
@@ -6525,7 +6525,7 @@
           <t>TOTAL GENERAL</t>
         </is>
       </c>
-      <c r="C26" s="145">
+      <c r="C26" s="141">
         <f>SUM(C18:C25)</f>
         <v/>
       </c>
@@ -6601,7 +6601,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="136" t="inlineStr">
+      <c r="B1" s="147" t="inlineStr">
         <is>
           <t>DETALLE ASESORES COMERCIALES</t>
         </is>
@@ -6617,47 +6617,47 @@
       </c>
     </row>
     <row r="5" ht="19.5" customHeight="1" s="137">
-      <c r="B5" s="145" t="inlineStr">
+      <c r="B5" s="141" t="inlineStr">
         <is>
           <t>Unidad de Negocio</t>
         </is>
       </c>
-      <c r="C5" s="145" t="inlineStr">
+      <c r="C5" s="141" t="inlineStr">
         <is>
           <t>Asesor</t>
         </is>
       </c>
-      <c r="D5" s="145" t="inlineStr">
+      <c r="D5" s="141" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="E5" s="145" t="inlineStr">
+      <c r="E5" s="141" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="F5" s="145" t="inlineStr">
+      <c r="F5" s="141" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="G5" s="145" t="inlineStr">
+      <c r="G5" s="141" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="H5" s="145" t="inlineStr">
+      <c r="H5" s="141" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="I5" s="145" t="inlineStr">
+      <c r="I5" s="141" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="J5" s="145" t="inlineStr">
+      <c r="J5" s="141" t="inlineStr">
         <is>
           <t>% Cumpl. Plan</t>
         </is>
@@ -6994,15 +6994,15 @@
         <f>E14/D14</f>
         <v/>
       </c>
-      <c r="G14" s="155">
+      <c r="G14" s="158">
         <f>SUM(G6:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="155">
+      <c r="H14" s="158">
         <f>SUM(H6:H13)</f>
         <v/>
       </c>
-      <c r="I14" s="155">
+      <c r="I14" s="158">
         <f>SUM(I6:I13)</f>
         <v/>
       </c>
@@ -7342,15 +7342,15 @@
         <f>E23/D23</f>
         <v/>
       </c>
-      <c r="G23" s="155">
+      <c r="G23" s="158">
         <f>SUM(G15:G22)</f>
         <v/>
       </c>
-      <c r="H23" s="155">
+      <c r="H23" s="158">
         <f>SUM(H15:H22)</f>
         <v/>
       </c>
-      <c r="I23" s="155">
+      <c r="I23" s="158">
         <f>SUM(I15:I22)</f>
         <v/>
       </c>
@@ -7690,15 +7690,15 @@
         <f>E32/D32</f>
         <v/>
       </c>
-      <c r="G32" s="155">
+      <c r="G32" s="158">
         <f>SUM(G24:G31)</f>
         <v/>
       </c>
-      <c r="H32" s="155">
+      <c r="H32" s="158">
         <f>SUM(H24:H31)</f>
         <v/>
       </c>
-      <c r="I32" s="155">
+      <c r="I32" s="158">
         <f>SUM(I24:I31)</f>
         <v/>
       </c>
@@ -8038,15 +8038,15 @@
         <f>E41/D41</f>
         <v/>
       </c>
-      <c r="G41" s="155">
+      <c r="G41" s="158">
         <f>SUM(G33:G40)</f>
         <v/>
       </c>
-      <c r="H41" s="155">
+      <c r="H41" s="158">
         <f>SUM(H33:H40)</f>
         <v/>
       </c>
-      <c r="I41" s="155">
+      <c r="I41" s="158">
         <f>SUM(I33:I40)</f>
         <v/>
       </c>
@@ -8113,15 +8113,15 @@
         <f>E43/D43</f>
         <v/>
       </c>
-      <c r="G43" s="155">
+      <c r="G43" s="158">
         <f>SUM(G42:G42)</f>
         <v/>
       </c>
-      <c r="H43" s="155">
+      <c r="H43" s="158">
         <f>SUM(H42:H42)</f>
         <v/>
       </c>
-      <c r="I43" s="155">
+      <c r="I43" s="158">
         <f>SUM(I42:I42)</f>
         <v/>
       </c>
@@ -8461,15 +8461,15 @@
         <f>E52/D52</f>
         <v/>
       </c>
-      <c r="G52" s="155">
+      <c r="G52" s="158">
         <f>SUM(G44:G51)</f>
         <v/>
       </c>
-      <c r="H52" s="155">
+      <c r="H52" s="158">
         <f>SUM(H44:H51)</f>
         <v/>
       </c>
-      <c r="I52" s="155">
+      <c r="I52" s="158">
         <f>SUM(I44:I51)</f>
         <v/>
       </c>
@@ -8575,15 +8575,15 @@
         <f>E55/D55</f>
         <v/>
       </c>
-      <c r="G55" s="155">
+      <c r="G55" s="158">
         <f>SUM(G53:G54)</f>
         <v/>
       </c>
-      <c r="H55" s="155">
+      <c r="H55" s="158">
         <f>SUM(H53:H54)</f>
         <v/>
       </c>
-      <c r="I55" s="155">
+      <c r="I55" s="158">
         <f>SUM(I53:I54)</f>
         <v/>
       </c>
@@ -8767,15 +8767,15 @@
         <f>E60/D60</f>
         <v/>
       </c>
-      <c r="G60" s="155">
+      <c r="G60" s="158">
         <f>SUM(G56:G59)</f>
         <v/>
       </c>
-      <c r="H60" s="155">
+      <c r="H60" s="158">
         <f>SUM(H56:H59)</f>
         <v/>
       </c>
-      <c r="I60" s="155">
+      <c r="I60" s="158">
         <f>SUM(I56:I59)</f>
         <v/>
       </c>
@@ -8803,11 +8803,11 @@
         <f>E61/D61</f>
         <v/>
       </c>
-      <c r="G61" s="145">
+      <c r="G61" s="141">
         <f>Datos!G50</f>
         <v/>
       </c>
-      <c r="H61" s="145">
+      <c r="H61" s="141">
         <f>Datos!F50</f>
         <v/>
       </c>
@@ -8850,7 +8850,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — SANIN</t>
         </is>
@@ -8867,41 +8867,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="159" t="inlineStr">
+      <c r="B6" s="167" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="165">
+      <c r="B7" s="155">
         <f>TEXT((Datos!D4+Datos!D5+Datos!D6+Datos!D7+Datos!D8+Datos!D9+Datos!D10+Datos!D11)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C4+Datos!C5+Datos!C6+Datos!C7+Datos!C8+Datos!C9+Datos!C10+Datos!C11)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D4+Datos!D5+Datos!D6+Datos!D7+Datos!D8+Datos!D9+Datos!D10+Datos!D11)/(Datos!C4+Datos!C5+Datos!C6+Datos!C7+Datos!C8+Datos!C9+Datos!C10+Datos!C11),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G4+Datos!G5+Datos!G6+Datos!G7+Datos!G8+Datos!G9+Datos!G10+Datos!G11)/(Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11),"0.0%")</f>
         <v/>
       </c>
@@ -8910,41 +8910,41 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
       </c>
-      <c r="F11" s="163" t="inlineStr">
+      <c r="F11" s="153" t="inlineStr">
         <is>
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G4+Datos!G5+Datos!G6+Datos!G7+Datos!G8+Datos!G9+Datos!G10+Datos!G11,"0")&amp;" / "&amp;TEXT(Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H4:H11,"&gt;="&amp;1),"0")&amp;" / "&amp;"8"</f>
         <v/>
       </c>
-      <c r="F12" s="171">
+      <c r="F12" s="163">
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B4:B11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0)),4))),MID(INDEX(Datos!B4:B11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0)),6,100),INDEX(Datos!B4:B11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11-Datos!G4+Datos!G5+Datos!G6+Datos!G7+Datos!G8+Datos!G9+Datos!G10+Datos!G11),"0")&amp;IF(Datos!G4+Datos!G5+Datos!G6+Datos!G7+Datos!G8+Datos!G9+Datos!G10+Datos!G11&gt;=Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -8953,49 +8953,49 @@
     <row r="14" ht="18" customHeight="1" s="137"/>
     <row r="15" ht="7.5" customHeight="1" s="137"/>
     <row r="16" ht="19.5" customHeight="1" s="137">
-      <c r="B16" s="164" t="inlineStr">
+      <c r="B16" s="154" t="inlineStr">
         <is>
           <t>DETALLE DE ASESORES — SANIN</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -9299,7 +9299,7 @@
         <f>Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11</f>
         <v/>
       </c>
-      <c r="H26" s="155">
+      <c r="H26" s="158">
         <f>SUM(H18:H25)</f>
         <v/>
       </c>
@@ -9310,32 +9310,32 @@
     </row>
     <row r="27" ht="7.5" customHeight="1" s="137"/>
     <row r="28" ht="18" customHeight="1" s="137">
-      <c r="B28" s="158" t="inlineStr">
+      <c r="B28" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="137">
-      <c r="B29" s="156">
+      <c r="B29" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D4+Datos!D5+Datos!D6+Datos!D7+Datos!D8+Datos!D9+Datos!D10+Datos!D11)/(Datos!C4+Datos!C5+Datos!C6+Datos!C7+Datos!C8+Datos!C9+Datos!C10+Datos!C11),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="137">
-      <c r="B30" s="153">
+      <c r="B30" s="170">
         <f>IF(COUNTIF(Datos!H4:H11,"&gt;="&amp;1)=8,"✔ "&amp;8&amp;" de 8 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G4+Datos!G5+Datos!G6+Datos!G7+Datos!G8+Datos!G9+Datos!G10+Datos!G11)-(Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H4:H11,"&gt;="&amp;1)&amp;" de 8 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F4+Datos!F5+Datos!F6+Datos!F7+Datos!F8+Datos!F9+Datos!F10+Datos!F11)-(Datos!G4+Datos!G5+Datos!G6+Datos!G7+Datos!G8+Datos!G9+Datos!G10+Datos!G11))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="137">
-      <c r="B31" s="156">
+      <c r="B31" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B4:B11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0)),4))),MID(INDEX(Datos!B4:B11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0)),6,100),INDEX(Datos!B4:B11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0)))&amp;" con "&amp;TEXT(MAX(Datos!D4:D11),"$#,##0")&amp;" y "&amp;INDEX(Datos!G4:G11,MATCH(MAX(Datos!D4:D11),Datos!D4:D11,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="137">
-      <c r="B32" s="153">
+      <c r="B32" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B4:B11,MATCH(MIN(Datos!D4:D11),Datos!D4:D11,0)),4))),MID(INDEX(Datos!B4:B11,MATCH(MIN(Datos!D4:D11),Datos!D4:D11,0)),6,100),INDEX(Datos!B4:B11,MATCH(MIN(Datos!D4:D11),Datos!D4:D11,0)))&amp;" con "&amp;TEXT(MIN(Datos!D4:D11),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E4:E11),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -9361,8 +9361,8 @@
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="H7:I9"/>
+    <mergeCell ref="D12:E14"/>
     <mergeCell ref="B30:I30"/>
-    <mergeCell ref="D12:E14"/>
     <mergeCell ref="H12:I14"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B4:I4"/>
@@ -9392,7 +9392,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — CASA LUKER</t>
         </is>
@@ -9409,41 +9409,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="169" t="inlineStr">
+      <c r="B6" s="161" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="160">
+      <c r="B7" s="168">
         <f>TEXT((Datos!D20+Datos!D21+Datos!D22+Datos!D23+Datos!D24+Datos!D25+Datos!D26+Datos!D27)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C20+Datos!C21+Datos!C22+Datos!C23+Datos!C24+Datos!C25+Datos!C26+Datos!C27)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D20+Datos!D21+Datos!D22+Datos!D23+Datos!D24+Datos!D25+Datos!D26+Datos!D27)/(Datos!C20+Datos!C21+Datos!C22+Datos!C23+Datos!C24+Datos!C25+Datos!C26+Datos!C27),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G20+Datos!G21+Datos!G22+Datos!G23+Datos!G24+Datos!G25+Datos!G26+Datos!G27)/(Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27),"0.0%")</f>
         <v/>
       </c>
@@ -9452,12 +9452,12 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
@@ -9467,18 +9467,18 @@
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G20+Datos!G21+Datos!G22+Datos!G23+Datos!G24+Datos!G25+Datos!G26+Datos!G27,"0")&amp;" / "&amp;TEXT(Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H20:H27,"&gt;="&amp;1),"0")&amp;" / "&amp;"8"</f>
         <v/>
       </c>
@@ -9486,7 +9486,7 @@
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B20:B27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0)),4))),MID(INDEX(Datos!B20:B27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0)),6,100),INDEX(Datos!B20:B27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27-Datos!G20+Datos!G21+Datos!G22+Datos!G23+Datos!G24+Datos!G25+Datos!G26+Datos!G27),"0")&amp;IF(Datos!G20+Datos!G21+Datos!G22+Datos!G23+Datos!G24+Datos!G25+Datos!G26+Datos!G27&gt;=Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -9502,42 +9502,42 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -9841,7 +9841,7 @@
         <f>Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27</f>
         <v/>
       </c>
-      <c r="H26" s="155">
+      <c r="H26" s="158">
         <f>SUM(H18:H25)</f>
         <v/>
       </c>
@@ -9852,32 +9852,32 @@
     </row>
     <row r="27" ht="7.5" customHeight="1" s="137"/>
     <row r="28" ht="18" customHeight="1" s="137">
-      <c r="B28" s="158" t="inlineStr">
+      <c r="B28" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="137">
-      <c r="B29" s="156">
+      <c r="B29" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D20+Datos!D21+Datos!D22+Datos!D23+Datos!D24+Datos!D25+Datos!D26+Datos!D27)/(Datos!C20+Datos!C21+Datos!C22+Datos!C23+Datos!C24+Datos!C25+Datos!C26+Datos!C27),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="137">
-      <c r="B30" s="153">
+      <c r="B30" s="170">
         <f>IF(COUNTIF(Datos!H20:H27,"&gt;="&amp;1)=8,"✔ "&amp;8&amp;" de 8 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G20+Datos!G21+Datos!G22+Datos!G23+Datos!G24+Datos!G25+Datos!G26+Datos!G27)-(Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H20:H27,"&gt;="&amp;1)&amp;" de 8 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F20+Datos!F21+Datos!F22+Datos!F23+Datos!F24+Datos!F25+Datos!F26+Datos!F27)-(Datos!G20+Datos!G21+Datos!G22+Datos!G23+Datos!G24+Datos!G25+Datos!G26+Datos!G27))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="137">
-      <c r="B31" s="156">
+      <c r="B31" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B20:B27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0)),4))),MID(INDEX(Datos!B20:B27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0)),6,100),INDEX(Datos!B20:B27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0)))&amp;" con "&amp;TEXT(MAX(Datos!D20:D27),"$#,##0")&amp;" y "&amp;INDEX(Datos!G20:G27,MATCH(MAX(Datos!D20:D27),Datos!D20:D27,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="137">
-      <c r="B32" s="153">
+      <c r="B32" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B20:B27,MATCH(MIN(Datos!D20:D27),Datos!D20:D27,0)),4))),MID(INDEX(Datos!B20:B27,MATCH(MIN(Datos!D20:D27),Datos!D20:D27,0)),6,100),INDEX(Datos!B20:B27,MATCH(MIN(Datos!D20:D27),Datos!D20:D27,0)))&amp;" con "&amp;TEXT(MIN(Datos!D20:D27),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E20:E27),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -9903,8 +9903,8 @@
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="H7:I9"/>
+    <mergeCell ref="D12:E14"/>
     <mergeCell ref="B30:I30"/>
-    <mergeCell ref="D12:E14"/>
     <mergeCell ref="H12:I14"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B4:I4"/>
@@ -9934,7 +9934,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — COLOMBINA</t>
         </is>
@@ -9951,22 +9951,22 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="170" t="inlineStr">
+      <c r="B6" s="162" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
@@ -9977,15 +9977,15 @@
         <f>TEXT((Datos!D12+Datos!D13+Datos!D14+Datos!D15+Datos!D16+Datos!D17+Datos!D18+Datos!D19)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C12+Datos!C13+Datos!C14+Datos!C15+Datos!C16+Datos!C17+Datos!C18+Datos!C19)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D12+Datos!D13+Datos!D14+Datos!D15+Datos!D16+Datos!D17+Datos!D18+Datos!D19)/(Datos!C12+Datos!C13+Datos!C14+Datos!C15+Datos!C16+Datos!C17+Datos!C18+Datos!C19),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G12+Datos!G13+Datos!G14+Datos!G15+Datos!G16+Datos!G17+Datos!G18+Datos!G19)/(Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19),"0.0%")</f>
         <v/>
       </c>
@@ -9994,12 +9994,12 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
@@ -10009,26 +10009,26 @@
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G12+Datos!G13+Datos!G14+Datos!G15+Datos!G16+Datos!G17+Datos!G18+Datos!G19,"0")&amp;" / "&amp;TEXT(Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H12:H19,"&gt;="&amp;1),"0")&amp;" / "&amp;"8"</f>
         <v/>
       </c>
-      <c r="F12" s="168">
+      <c r="F12" s="160">
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B12:B19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0)),4))),MID(INDEX(Datos!B12:B19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0)),6,100),INDEX(Datos!B12:B19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19-Datos!G12+Datos!G13+Datos!G14+Datos!G15+Datos!G16+Datos!G17+Datos!G18+Datos!G19),"0")&amp;IF(Datos!G12+Datos!G13+Datos!G14+Datos!G15+Datos!G16+Datos!G17+Datos!G18+Datos!G19&gt;=Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -10044,42 +10044,42 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -10383,7 +10383,7 @@
         <f>Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19</f>
         <v/>
       </c>
-      <c r="H26" s="155">
+      <c r="H26" s="158">
         <f>SUM(H18:H25)</f>
         <v/>
       </c>
@@ -10394,32 +10394,32 @@
     </row>
     <row r="27" ht="7.5" customHeight="1" s="137"/>
     <row r="28" ht="18" customHeight="1" s="137">
-      <c r="B28" s="158" t="inlineStr">
+      <c r="B28" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="137">
-      <c r="B29" s="156">
+      <c r="B29" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D12+Datos!D13+Datos!D14+Datos!D15+Datos!D16+Datos!D17+Datos!D18+Datos!D19)/(Datos!C12+Datos!C13+Datos!C14+Datos!C15+Datos!C16+Datos!C17+Datos!C18+Datos!C19),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="137">
-      <c r="B30" s="153">
+      <c r="B30" s="170">
         <f>IF(COUNTIF(Datos!H12:H19,"&gt;="&amp;1)=8,"✔ "&amp;8&amp;" de 8 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G12+Datos!G13+Datos!G14+Datos!G15+Datos!G16+Datos!G17+Datos!G18+Datos!G19)-(Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H12:H19,"&gt;="&amp;1)&amp;" de 8 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F12+Datos!F13+Datos!F14+Datos!F15+Datos!F16+Datos!F17+Datos!F18+Datos!F19)-(Datos!G12+Datos!G13+Datos!G14+Datos!G15+Datos!G16+Datos!G17+Datos!G18+Datos!G19))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="137">
-      <c r="B31" s="156">
+      <c r="B31" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B12:B19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0)),4))),MID(INDEX(Datos!B12:B19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0)),6,100),INDEX(Datos!B12:B19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0)))&amp;" con "&amp;TEXT(MAX(Datos!D12:D19),"$#,##0")&amp;" y "&amp;INDEX(Datos!G12:G19,MATCH(MAX(Datos!D12:D19),Datos!D12:D19,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="137">
-      <c r="B32" s="153">
+      <c r="B32" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B12:B19,MATCH(MIN(Datos!D12:D19),Datos!D12:D19,0)),4))),MID(INDEX(Datos!B12:B19,MATCH(MIN(Datos!D12:D19),Datos!D12:D19,0)),6,100),INDEX(Datos!B12:B19,MATCH(MIN(Datos!D12:D19),Datos!D12:D19,0)))&amp;" con "&amp;TEXT(MIN(Datos!D12:D19),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E12:E19),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -10445,8 +10445,8 @@
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="H7:I9"/>
+    <mergeCell ref="D12:E14"/>
     <mergeCell ref="B30:I30"/>
-    <mergeCell ref="D12:E14"/>
     <mergeCell ref="H12:I14"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B4:I4"/>
@@ -10476,7 +10476,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — TECNOQUIMICAS</t>
         </is>
@@ -10493,41 +10493,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="166" t="inlineStr">
+      <c r="B6" s="156" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="167">
+      <c r="B7" s="159">
         <f>TEXT((Datos!D28+Datos!D29+Datos!D30+Datos!D31+Datos!D32+Datos!D33+Datos!D34+Datos!D35)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C28+Datos!C29+Datos!C30+Datos!C31+Datos!C32+Datos!C33+Datos!C34+Datos!C35)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D28+Datos!D29+Datos!D30+Datos!D31+Datos!D32+Datos!D33+Datos!D34+Datos!D35)/(Datos!C28+Datos!C29+Datos!C30+Datos!C31+Datos!C32+Datos!C33+Datos!C34+Datos!C35),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G28+Datos!G29+Datos!G30+Datos!G31+Datos!G32+Datos!G33+Datos!G34+Datos!G35)/(Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35),"0.0%")</f>
         <v/>
       </c>
@@ -10536,12 +10536,12 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
@@ -10551,26 +10551,26 @@
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G28+Datos!G29+Datos!G30+Datos!G31+Datos!G32+Datos!G33+Datos!G34+Datos!G35,"0")&amp;" / "&amp;TEXT(Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H28:H35,"&gt;="&amp;1),"0")&amp;" / "&amp;"8"</f>
         <v/>
       </c>
-      <c r="F12" s="161">
+      <c r="F12" s="169">
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B28:B35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0)),4))),MID(INDEX(Datos!B28:B35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0)),6,100),INDEX(Datos!B28:B35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35-Datos!G28+Datos!G29+Datos!G30+Datos!G31+Datos!G32+Datos!G33+Datos!G34+Datos!G35),"0")&amp;IF(Datos!G28+Datos!G29+Datos!G30+Datos!G31+Datos!G32+Datos!G33+Datos!G34+Datos!G35&gt;=Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -10586,42 +10586,42 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -10925,7 +10925,7 @@
         <f>Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35</f>
         <v/>
       </c>
-      <c r="H26" s="155">
+      <c r="H26" s="158">
         <f>SUM(H18:H25)</f>
         <v/>
       </c>
@@ -10936,32 +10936,32 @@
     </row>
     <row r="27" ht="7.5" customHeight="1" s="137"/>
     <row r="28" ht="18" customHeight="1" s="137">
-      <c r="B28" s="158" t="inlineStr">
+      <c r="B28" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="137">
-      <c r="B29" s="156">
+      <c r="B29" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D28+Datos!D29+Datos!D30+Datos!D31+Datos!D32+Datos!D33+Datos!D34+Datos!D35)/(Datos!C28+Datos!C29+Datos!C30+Datos!C31+Datos!C32+Datos!C33+Datos!C34+Datos!C35),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="137">
-      <c r="B30" s="153">
+      <c r="B30" s="170">
         <f>IF(COUNTIF(Datos!H28:H35,"&gt;="&amp;1)=8,"✔ "&amp;8&amp;" de 8 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G28+Datos!G29+Datos!G30+Datos!G31+Datos!G32+Datos!G33+Datos!G34+Datos!G35)-(Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H28:H35,"&gt;="&amp;1)&amp;" de 8 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F28+Datos!F29+Datos!F30+Datos!F31+Datos!F32+Datos!F33+Datos!F34+Datos!F35)-(Datos!G28+Datos!G29+Datos!G30+Datos!G31+Datos!G32+Datos!G33+Datos!G34+Datos!G35))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="137">
-      <c r="B31" s="156">
+      <c r="B31" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B28:B35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0)),4))),MID(INDEX(Datos!B28:B35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0)),6,100),INDEX(Datos!B28:B35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0)))&amp;" con "&amp;TEXT(MAX(Datos!D28:D35),"$#,##0")&amp;" y "&amp;INDEX(Datos!G28:G35,MATCH(MAX(Datos!D28:D35),Datos!D28:D35,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="137">
-      <c r="B32" s="153">
+      <c r="B32" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B28:B35,MATCH(MIN(Datos!D28:D35),Datos!D28:D35,0)),4))),MID(INDEX(Datos!B28:B35,MATCH(MIN(Datos!D28:D35),Datos!D28:D35,0)),6,100),INDEX(Datos!B28:B35,MATCH(MIN(Datos!D28:D35),Datos!D28:D35,0)))&amp;" con "&amp;TEXT(MIN(Datos!D28:D35),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E28:E35),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -10987,8 +10987,8 @@
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="H7:I9"/>
+    <mergeCell ref="D12:E14"/>
     <mergeCell ref="B30:I30"/>
-    <mergeCell ref="D12:E14"/>
     <mergeCell ref="H12:I14"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B4:I4"/>
@@ -11018,7 +11018,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — CLIENTES ESPECIALES</t>
         </is>
@@ -11035,41 +11035,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="155" t="inlineStr">
+      <c r="B6" s="158" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="157">
+      <c r="B7" s="165">
         <f>TEXT((Datos!D36+Datos!#REF!)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C36+Datos!#REF!)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D36+Datos!#REF!)/(Datos!C36+Datos!#REF!),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G36+Datos!#REF!)/(Datos!F36+Datos!#REF!),"0.0%")</f>
         <v/>
       </c>
@@ -11078,12 +11078,12 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
@@ -11093,18 +11093,18 @@
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G36+Datos!#REF!,"0")&amp;" / "&amp;TEXT(Datos!F36+Datos!#REF!,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H36:H36,"&gt;="&amp;1),"0")&amp;" / "&amp;"2"</f>
         <v/>
       </c>
@@ -11112,7 +11112,7 @@
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B36:B36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0)),4))),MID(INDEX(Datos!B36:B36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0)),6,100),INDEX(Datos!B36:B36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F36+Datos!#REF!-Datos!G36+Datos!#REF!),"0")&amp;IF(Datos!G36+Datos!#REF!&gt;=Datos!F36+Datos!#REF!," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -11128,42 +11128,42 @@
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -11263,7 +11263,7 @@
         <f>Datos!F36+Datos!#REF!</f>
         <v/>
       </c>
-      <c r="H20" s="155">
+      <c r="H20" s="158">
         <f>SUM(H18:H19)</f>
         <v/>
       </c>
@@ -11274,32 +11274,32 @@
     </row>
     <row r="21" ht="7.5" customHeight="1" s="137"/>
     <row r="22" ht="18" customHeight="1" s="137">
-      <c r="B22" s="158" t="inlineStr">
+      <c r="B22" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="137">
-      <c r="B23" s="156">
+      <c r="B23" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D36+Datos!#REF!)/(Datos!C36+Datos!#REF!),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="137">
-      <c r="B24" s="153">
+      <c r="B24" s="170">
         <f>IF(COUNTIF(Datos!H36:H36,"&gt;="&amp;1)=2,"✔ "&amp;2&amp;" de 2 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G36+Datos!#REF!)-(Datos!F36+Datos!#REF!))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H36:H36,"&gt;="&amp;1)&amp;" de 2 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F36+Datos!#REF!)-(Datos!G36+Datos!#REF!))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="137">
-      <c r="B25" s="156">
+      <c r="B25" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B36:B36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0)),4))),MID(INDEX(Datos!B36:B36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0)),6,100),INDEX(Datos!B36:B36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0)))&amp;" con "&amp;TEXT(MAX(Datos!D36:D36),"$#,##0")&amp;" y "&amp;INDEX(Datos!G36:G36,MATCH(MAX(Datos!D36:D36),Datos!D36:D36,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="137">
-      <c r="B26" s="153">
+      <c r="B26" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B36:B36,MATCH(MIN(Datos!D36:D36),Datos!D36:D36,0)),4))),MID(INDEX(Datos!B36:B36,MATCH(MIN(Datos!D36:D36),Datos!D36:D36,0)),6,100),INDEX(Datos!B36:B36,MATCH(MIN(Datos!D36:D36),Datos!D36:D36,0)))&amp;" con "&amp;TEXT(MIN(Datos!D36:D36),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E36:E36),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -11356,7 +11356,7 @@
   </cols>
   <sheetData>
     <row r="1" ht="12" customHeight="1" s="137">
-      <c r="B1" s="154" t="inlineStr">
+      <c r="B1" s="164" t="inlineStr">
         <is>
           <t>UNIDAD DE NEGOCIO — BRINSA</t>
         </is>
@@ -11373,41 +11373,41 @@
     </row>
     <row r="5" ht="7.5" customHeight="1" s="137"/>
     <row r="6" ht="18" customHeight="1" s="137">
-      <c r="B6" s="183" t="inlineStr">
+      <c r="B6" s="187" t="inlineStr">
         <is>
           <t>VENTA DÍA</t>
         </is>
       </c>
-      <c r="D6" s="155" t="inlineStr">
+      <c r="D6" s="158" t="inlineStr">
         <is>
           <t>PRESUPUESTO DÍA</t>
         </is>
       </c>
-      <c r="F6" s="166" t="inlineStr">
+      <c r="F6" s="156" t="inlineStr">
         <is>
           <t>% CUMPL. PPTO</t>
         </is>
       </c>
-      <c r="H6" s="169" t="inlineStr">
+      <c r="H6" s="161" t="inlineStr">
         <is>
           <t>% CUMPL. PLAN</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="137">
-      <c r="B7" s="186">
+      <c r="B7" s="185">
         <f>TEXT((Datos!D37+Datos!D38+Datos!D39+Datos!D40+Datos!D41+Datos!D42+Datos!D43+Datos!D44)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="D7" s="157">
+      <c r="D7" s="165">
         <f>TEXT((Datos!C37+Datos!C38+Datos!C39+Datos!C40+Datos!C41+Datos!C42+Datos!C43+Datos!C44)/1000000,"$#,##0.00")&amp;"M"</f>
         <v/>
       </c>
-      <c r="F7" s="167">
+      <c r="F7" s="159">
         <f>TEXT((Datos!D37+Datos!D38+Datos!D39+Datos!D40+Datos!D41+Datos!D42+Datos!D43+Datos!D44)/(Datos!C37+Datos!C38+Datos!C39+Datos!C40+Datos!C41+Datos!C42+Datos!C43+Datos!C44),"0.0%")</f>
         <v/>
       </c>
-      <c r="H7" s="160">
+      <c r="H7" s="168">
         <f>TEXT((Datos!G37+Datos!G38+Datos!G39+Datos!G40+Datos!G41+Datos!G42+Datos!G43+Datos!G44)/(Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44),"0.0%")</f>
         <v/>
       </c>
@@ -11416,41 +11416,41 @@
     <row r="9" ht="18" customHeight="1" s="137"/>
     <row r="10" ht="7.5" customHeight="1" s="137"/>
     <row r="11" ht="18" customHeight="1" s="137">
-      <c r="B11" s="170" t="inlineStr">
+      <c r="B11" s="162" t="inlineStr">
         <is>
           <t>FACTURAS / OBJETIVO</t>
         </is>
       </c>
-      <c r="D11" s="166" t="inlineStr">
+      <c r="D11" s="156" t="inlineStr">
         <is>
           <t>CUMPLEN META PLAN</t>
         </is>
       </c>
-      <c r="F11" s="184" t="inlineStr">
+      <c r="F11" s="183" t="inlineStr">
         <is>
           <t>MEJOR ASESOR</t>
         </is>
       </c>
-      <c r="H11" s="155" t="inlineStr">
+      <c r="H11" s="158" t="inlineStr">
         <is>
           <t>PEDIDOS FALTANTES</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="137">
-      <c r="B12" s="168">
+      <c r="B12" s="160">
         <f>TEXT(Datos!G37+Datos!G38+Datos!G39+Datos!G40+Datos!G41+Datos!G42+Datos!G43+Datos!G44,"0")&amp;" / "&amp;TEXT(Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44,"0")</f>
         <v/>
       </c>
-      <c r="D12" s="161">
+      <c r="D12" s="169">
         <f>TEXT(COUNTIF(Datos!H37:H44,"&gt;="&amp;1),"0")&amp;" / "&amp;"8"</f>
         <v/>
       </c>
-      <c r="F12" s="187">
+      <c r="F12" s="186">
         <f>IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B37:B44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0)),4))),MID(INDEX(Datos!B37:B44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0)),6,100),INDEX(Datos!B37:B44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0)))</f>
         <v/>
       </c>
-      <c r="H12" s="162">
+      <c r="H12" s="171">
         <f>TEXT(ABS(Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44-Datos!G37+Datos!G38+Datos!G39+Datos!G40+Datos!G41+Datos!G42+Datos!G43+Datos!G44),"0")&amp;IF(Datos!G37+Datos!G38+Datos!G39+Datos!G40+Datos!G41+Datos!G42+Datos!G43+Datos!G44&gt;=Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44," excedente"," pedidos")</f>
         <v/>
       </c>
@@ -11459,49 +11459,49 @@
     <row r="14" ht="18" customHeight="1" s="137"/>
     <row r="15" ht="7.5" customHeight="1" s="137"/>
     <row r="16" ht="19.5" customHeight="1" s="137">
-      <c r="B16" s="185" t="inlineStr">
+      <c r="B16" s="184" t="inlineStr">
         <is>
           <t>DETALLE DE ASESORES — BRINSA</t>
         </is>
       </c>
     </row>
     <row r="17" ht="19.5" customHeight="1" s="137">
-      <c r="B17" s="159" t="inlineStr">
+      <c r="B17" s="167" t="inlineStr">
         <is>
           <t>Asesor Comercial</t>
         </is>
       </c>
-      <c r="C17" s="159" t="inlineStr">
+      <c r="C17" s="167" t="inlineStr">
         <is>
           <t>Ppto Día ($)</t>
         </is>
       </c>
-      <c r="D17" s="159" t="inlineStr">
+      <c r="D17" s="167" t="inlineStr">
         <is>
           <t>Venta Día ($)</t>
         </is>
       </c>
-      <c r="E17" s="159" t="inlineStr">
+      <c r="E17" s="167" t="inlineStr">
         <is>
           <t>% Cumpl. Ppto</t>
         </is>
       </c>
-      <c r="F17" s="159" t="inlineStr">
+      <c r="F17" s="167" t="inlineStr">
         <is>
           <t># Facturas</t>
         </is>
       </c>
-      <c r="G17" s="159" t="inlineStr">
+      <c r="G17" s="167" t="inlineStr">
         <is>
           <t>Obj. Plan</t>
         </is>
       </c>
-      <c r="H17" s="159" t="inlineStr">
+      <c r="H17" s="167" t="inlineStr">
         <is>
           <t>Faltante</t>
         </is>
       </c>
-      <c r="I17" s="159" t="inlineStr">
+      <c r="I17" s="167" t="inlineStr">
         <is>
           <t>Estado Plan</t>
         </is>
@@ -11805,7 +11805,7 @@
         <f>Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44</f>
         <v/>
       </c>
-      <c r="H26" s="155">
+      <c r="H26" s="158">
         <f>SUM(H18:H25)</f>
         <v/>
       </c>
@@ -11816,32 +11816,32 @@
     </row>
     <row r="27" ht="7.5" customHeight="1" s="137"/>
     <row r="28" ht="18" customHeight="1" s="137">
-      <c r="B28" s="158" t="inlineStr">
+      <c r="B28" s="166" t="inlineStr">
         <is>
           <t>ANÁLISIS DE GESTIÓN</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="137">
-      <c r="B29" s="156">
+      <c r="B29" s="157">
         <f>"▶ Venta del día en progreso: "&amp;TEXT((Datos!D37+Datos!D38+Datos!D39+Datos!D40+Datos!D41+Datos!D42+Datos!D43+Datos!D44)/(Datos!C37+Datos!C38+Datos!C39+Datos!C40+Datos!C41+Datos!C42+Datos!C43+Datos!C44),"0.0%")&amp;" del presupuesto."</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="137">
-      <c r="B30" s="153">
+      <c r="B30" s="170">
         <f>IF(COUNTIF(Datos!H37:H44,"&gt;="&amp;1)=8,"✔ "&amp;8&amp;" de 8 asesores cumplen meta. Excedente de "&amp;ABS((Datos!G37+Datos!G38+Datos!G39+Datos!G40+Datos!G41+Datos!G42+Datos!G43+Datos!G44)-(Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44))&amp;" pedidos sobre el objetivo.","▶ "&amp;COUNTIF(Datos!H37:H44,"&gt;="&amp;1)&amp;" de 8 asesores cumplen meta. Pendiente cerrar "&amp;MAX(0,(Datos!F37+Datos!F38+Datos!F39+Datos!F40+Datos!F41+Datos!F42+Datos!F43+Datos!F44)-(Datos!G37+Datos!G38+Datos!G39+Datos!G40+Datos!G41+Datos!G42+Datos!G43+Datos!G44))&amp;" pedidos.")</f>
         <v/>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="137">
-      <c r="B31" s="156">
+      <c r="B31" s="157">
         <f>"★ Mejor asesor: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B37:B44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0)),4))),MID(INDEX(Datos!B37:B44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0)),6,100),INDEX(Datos!B37:B44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0)))&amp;" con "&amp;TEXT(MAX(Datos!D37:D44),"$#,##0")&amp;" y "&amp;INDEX(Datos!G37:G44,MATCH(MAX(Datos!D37:D44),Datos!D37:D44,0))&amp;" facturas."</f>
         <v/>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="137">
-      <c r="B32" s="153">
+      <c r="B32" s="170">
         <f>"⚠ Asesor con menor venta: "&amp;IF(ISNUMBER(VALUE(LEFT(INDEX(Datos!B37:B44,MATCH(MIN(Datos!D37:D44),Datos!D37:D44,0)),4))),MID(INDEX(Datos!B37:B44,MATCH(MIN(Datos!D37:D44),Datos!D37:D44,0)),6,100),INDEX(Datos!B37:B44,MATCH(MIN(Datos!D37:D44),Datos!D37:D44,0)))&amp;" con "&amp;TEXT(MIN(Datos!D37:D44),"$#,##0")&amp;" ("&amp;TEXT(MIN(Datos!E37:E44),"0.0%")&amp;" del ppto)."</f>
         <v/>
       </c>
@@ -11867,8 +11867,8 @@
     <mergeCell ref="B28:I28"/>
     <mergeCell ref="B6:C6"/>
     <mergeCell ref="H7:I9"/>
+    <mergeCell ref="D12:E14"/>
     <mergeCell ref="B30:I30"/>
-    <mergeCell ref="D12:E14"/>
     <mergeCell ref="H12:I14"/>
     <mergeCell ref="B32:I32"/>
     <mergeCell ref="B4:I4"/>

</xml_diff>